<commit_message>
feat: cheaper free-tier AI (batch meal plans, video rewards, daily Meals ad)
- batch-meal-plans: tomorrow's free-user plans via Anthropic's Message
  Batches API (half price), stored only after the same USDA, allergy,
  restriction and diet checks as generate-meal-plan; translated into the
  new profiles.language; chunked, time-bounded processing
- Concise prompt and lower token cap for free plans; shared
  usda_food_cache for USDA's hourly limit
- Rewarded video adds 1 coach message and $0.006 of AI budget
- One interstitial when a free user first opens Meals each day
- Admin settings for the batch job and interstitial assumptions;
  spreadsheet, docs and decision log updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FhfEYVk2hN2wqZc7JaLb6E
</commit_message>
<xml_diff>
--- a/docs/business/ai-ad-economics.xlsx
+++ b/docs/business/ai-ad-economics.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -726,33 +726,37 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Translation (non-English) — input tokens</t>
+          <t>Free meal plan — output tokens (concise dishes)</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Dish texts sent back for translation</t>
+          <t>Free plans: shorter descriptions, 2–4 ingredients, 3 short steps; 1,000-token cap</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Translation (non-English) — output tokens</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="C20" s="7" t="inlineStr"/>
+          <t>Share of free plans made overnight by the batch job</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Active free users get tomorrow's plan from batch-meal-plans; the rest are made on demand</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Share of users not using English</t>
+          <t>Batch API discount</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
@@ -760,303 +764,317 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>German, French, Spanish, Italian, Greek</t>
+          <t>Anthropic Message Batches: 50% off input and output</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Another idea — input tokens</t>
+          <t>Translation (non-English) — input tokens</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="C22" s="7" t="inlineStr"/>
+        <v>800</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Dish texts sent back for translation</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Another idea — output tokens</t>
+          <t>Translation (non-English) — output tokens</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="C23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Another idea — attempts</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C24" s="7" t="inlineStr"/>
+          <t>Share of users not using English</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>German, French, Spanish, Italian, Greek</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Food photo scan — input tokens</t>
+          <t>Another idea — input tokens</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>2300</v>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Image ~1,500 + prompt</t>
-        </is>
-      </c>
+        <v>1800</v>
+      </c>
+      <c r="C25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Food photo scan — output tokens</t>
+          <t>Another idea — output tokens</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="C26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Food photo scan — attempts</t>
+          <t>Another idea — attempts</t>
         </is>
       </c>
       <c r="B27" s="10" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="C27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Ads (AdMob, EU; estimates)</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Food photo scan — input tokens</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>2300</v>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Image ~1,500 + prompt</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Banner eCPM (USD per 1,000 impressions)</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Assumption: EU banners typically $0.3–1.0</t>
-        </is>
-      </c>
+          <t>Food photo scan — output tokens</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="C29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Banner impressions per active day</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Home + Progress banners with refresh</t>
-        </is>
-      </c>
+          <t>Food photo scan — attempts</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Rewarded video eCPM (USD per 1,000 views)</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Assumption: EU rewarded typically $6–15</t>
-        </is>
-      </c>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Ads (AdMob, EU; estimates)</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Share of impressions non-personalised</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="n">
-        <v>0.6</v>
+          <t>Banner eCPM (USD per 1,000 impressions)</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>0.5</v>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>All iOS (no ATT) + EU users who decline consent</t>
+          <t>Assumption: EU banners typically $0.3–1.0</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Non-personalised earnings vs personalised</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="n">
-        <v>0.6</v>
+          <t>Banner impressions per active day</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>15</v>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>NPA ads typically earn 30–50% less</t>
+          <t>Home + Progress banners with refresh</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Free-tier limits and budget (app_config)</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Rewarded video eCPM (USD per 1,000 views)</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Assumption: EU rewarded typically $6–15</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Base AI budget per day (USD)</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="n">
-        <v>0.04</v>
+          <t>Interstitial eCPM (USD per 1,000 impressions)</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>ai_free_daily_budget_usd: a backstop sized to the free allowance</t>
+          <t>Assumption: EU interstitials typically $2–6</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Extra AI budget per rewarded video (USD)</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="n">
-        <v>0.01</v>
+          <t>Interstitials per active day</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>ai_budget_per_boost_usd: the cost of what a video adds</t>
+          <t>Once a day on first opening Meals (not on the onboarding day)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Rewarded videos per day that count (max)</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="n">
-        <v>3</v>
+          <t>Share of impressions non-personalised</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>0.6</v>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>ai_boosts_daily_max</t>
+          <t>All iOS (no ATT) + EU users who decline consent</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Usage per active day — typical free user</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Non-personalised earnings vs personalised</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>NPA ads typically earn 30–50% less</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Meal plans</t>
-        </is>
-      </c>
-      <c r="B39" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Today's plan is always made</t>
-        </is>
-      </c>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Free-tier limits and budget (app_config)</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Coach messages</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" s="7" t="inlineStr"/>
+          <t>Base AI budget per day (USD)</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>ai_free_daily_budget_usd: a backstop sized to the free allowance</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Another idea</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C41" s="7" t="inlineStr"/>
+          <t>Extra AI budget per rewarded video (USD)</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>ai_budget_per_boost_usd: about what a rewarded video earns after the NPA discount</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Food photo scans</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C42" s="7" t="inlineStr"/>
+          <t>Rewarded videos per day that count (max)</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>ai_boosts_daily_max</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Rewarded videos watched</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Meal reveals + AI boosts</t>
-        </is>
-      </c>
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Usage per active day — typical free user</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Usage per active day — heavy free user</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Meal plans</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Today's plan is always made</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Meal plans</t>
+          <t>Coach messages</t>
         </is>
       </c>
       <c r="B45" s="10" t="n">
@@ -1067,207 +1085,264 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Coach messages</t>
+          <t>Another idea</t>
         </is>
       </c>
       <c r="B46" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>3 free + 3 per video x 3</t>
-        </is>
-      </c>
+        <v>0.3</v>
+      </c>
+      <c r="C46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Another idea</t>
+          <t>Food photo scans</t>
         </is>
       </c>
       <c r="B47" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>1 free + 1 per video x 3</t>
-        </is>
-      </c>
+        <v>0.3</v>
+      </c>
+      <c r="C47" s="7" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Food photo scans</t>
+          <t>Rewarded videos watched</t>
         </is>
       </c>
       <c r="B48" s="10" t="n">
-        <v>4</v>
+        <v>1.2</v>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>1 free + 1 per video x 3</t>
+          <t>Meal reveals + AI boosts</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Rewarded videos watched</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>The daily maximum that counts</t>
-        </is>
-      </c>
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Usage per active day — heavy free user</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Engagement and other costs</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Meal plans</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Active days per month (free user)</t>
+          <t>Coach messages</t>
         </is>
       </c>
       <c r="B51" s="10" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Typical after the first weeks</t>
+          <t>3 free + 1 per video x 3</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure per user per month (USD)</t>
-        </is>
-      </c>
-      <c r="B52" s="11" t="n">
-        <v>0.01</v>
+          <t>Another idea</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Supabase, push, Sentry/PostHog shared across ~10k MAU</t>
+          <t>1 free + 1 per video x 3</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>SMS code cost per phone sign-up (USD)</t>
-        </is>
-      </c>
-      <c r="B53" s="11" t="n">
-        <v>0.05</v>
+          <t>Food photo scans</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>sms.to EU, about EUR 0.03–0.08; email sign-up ~0</t>
+          <t>1 free + 1 per video x 3</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rewarded videos watched</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>The daily maximum that counts</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Premium price per month (USD)</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="C55" s="7" t="inlineStr">
-        <is>
-          <t>Monthly plan (CLAUDE.md section 12)</t>
-        </is>
-      </c>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Engagement and other costs</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Store fee</t>
-        </is>
-      </c>
-      <c r="B56" s="9" t="n">
-        <v>0.15</v>
+          <t>Active days per month (free user)</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="n">
+        <v>12</v>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>App Store / Play small-business rate</t>
+          <t>Typical after the first weeks</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Conversion to Premium (share of monthly users)</t>
-        </is>
-      </c>
-      <c r="B57" s="9" t="n">
-        <v>0.03</v>
+          <t>Infrastructure per user per month (USD)</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="n">
+        <v>0.01</v>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Assumption: 2–5% is common</t>
+          <t>Supabase, push, Sentry/PostHog shared across ~10k MAU</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Premium active days per month</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C58" s="7" t="inlineStr"/>
+          <t>SMS code cost per phone sign-up (USD)</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>sms.to EU, about EUR 0.03–0.08; email sign-up ~0</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Premium coach messages per active day</t>
-        </is>
-      </c>
-      <c r="B59" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>Fair-use cap is 60</t>
-        </is>
-      </c>
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
+          <t>Premium price per month (USD)</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Monthly plan (CLAUDE.md section 12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Store fee</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>App Store / Play small-business rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Conversion to Premium (share of monthly users)</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Assumption: 2–5% is common</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Premium active days per month</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Premium coach messages per active day</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Fair-use cap is 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
           <t>Premium other AI per active day (USD)</t>
         </is>
       </c>
-      <c r="B60" s="11" t="n">
+      <c r="B65" s="11" t="n">
         <v>0.03</v>
       </c>
-      <c r="C60" s="7" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>Meal plan, insights, grocery, photos on Sonnet</t>
         </is>
@@ -1358,7 +1433,7 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>Assumptions!$B$18*(Assumptions!$B$16*(1-0)*Assumptions!$B$5+Assumptions!$B$16*0*Assumptions!$B$7+Assumptions!$B$17*Assumptions!$B$6)/1000000</f>
+        <f>Assumptions!$B$18*(Assumptions!$B$16*(1-0)*Assumptions!$B$5+Assumptions!$B$16*0*Assumptions!$B$7+Assumptions!$B$19*Assumptions!$B$6)/1000000*(1-Assumptions!$B$20*Assumptions!$B$21)</f>
         <v/>
       </c>
       <c r="C5" s="12">
@@ -1367,7 +1442,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>x attempts</t>
+          <t>free: concise output, part via the Batch API at half price; x attempts</t>
         </is>
       </c>
     </row>
@@ -1378,11 +1453,11 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>Assumptions!$B$21*(Assumptions!$B$19*Assumptions!$B$5+Assumptions!$B$20*Assumptions!$B$6)/1000000</f>
+        <f>Assumptions!$B$24*(Assumptions!$B$22*Assumptions!$B$5+Assumptions!$B$23*Assumptions!$B$6)/1000000</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>Assumptions!$B$21*(Assumptions!$B$19*Assumptions!$B$8+Assumptions!$B$20*Assumptions!$B$9)/1000000</f>
+        <f>Assumptions!$B$24*(Assumptions!$B$22*Assumptions!$B$8+Assumptions!$B$23*Assumptions!$B$9)/1000000</f>
         <v/>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -1398,11 +1473,11 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>Assumptions!$B$24*(Assumptions!$B$22*(1-0)*Assumptions!$B$5+Assumptions!$B$22*0*Assumptions!$B$7+Assumptions!$B$23*Assumptions!$B$6)/1000000</f>
+        <f>Assumptions!$B$27*(Assumptions!$B$25*(1-0)*Assumptions!$B$5+Assumptions!$B$25*0*Assumptions!$B$7+Assumptions!$B$26*Assumptions!$B$6)/1000000</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>Assumptions!$B$24*(Assumptions!$B$22*(1-0)*Assumptions!$B$8+Assumptions!$B$22*0*Assumptions!$B$10+Assumptions!$B$23*Assumptions!$B$9)/1000000</f>
+        <f>Assumptions!$B$27*(Assumptions!$B$25*(1-0)*Assumptions!$B$8+Assumptions!$B$25*0*Assumptions!$B$10+Assumptions!$B$26*Assumptions!$B$9)/1000000</f>
         <v/>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1418,11 +1493,11 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>Assumptions!$B$27*(Assumptions!$B$25*(1-0)*Assumptions!$B$5+Assumptions!$B$25*0*Assumptions!$B$7+Assumptions!$B$26*Assumptions!$B$6)/1000000</f>
+        <f>Assumptions!$B$30*(Assumptions!$B$28*(1-0)*Assumptions!$B$5+Assumptions!$B$28*0*Assumptions!$B$7+Assumptions!$B$29*Assumptions!$B$6)/1000000</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>Assumptions!$B$27*(Assumptions!$B$25*(1-0)*Assumptions!$B$8+Assumptions!$B$25*0*Assumptions!$B$10+Assumptions!$B$26*Assumptions!$B$9)/1000000</f>
+        <f>Assumptions!$B$30*(Assumptions!$B$28*(1-0)*Assumptions!$B$8+Assumptions!$B$28*0*Assumptions!$B$10+Assumptions!$B$29*Assumptions!$B$9)/1000000</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -1442,7 +1517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1484,11 +1559,11 @@
         </is>
       </c>
       <c r="B4" s="13">
-        <f>Assumptions!$B$30*Assumptions!$B$29/1000*(1-Assumptions!$B$32*(1-Assumptions!$B$33))</f>
+        <f>Assumptions!$B$33*Assumptions!$B$32/1000*(1-Assumptions!$B$37*(1-Assumptions!$B$38))</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>Assumptions!$B$30*Assumptions!$B$29/1000*(1-Assumptions!$B$32*(1-Assumptions!$B$33))</f>
+        <f>Assumptions!$B$33*Assumptions!$B$32/1000*(1-Assumptions!$B$37*(1-Assumptions!$B$38))</f>
         <v/>
       </c>
     </row>
@@ -1499,200 +1574,215 @@
         </is>
       </c>
       <c r="B5" s="13">
-        <f>Assumptions!$B$43*Assumptions!$B$31/1000*(1-Assumptions!$B$32*(1-Assumptions!$B$33))</f>
+        <f>Assumptions!$B$48*Assumptions!$B$34/1000*(1-Assumptions!$B$37*(1-Assumptions!$B$38))</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>Assumptions!$B$49*Assumptions!$B$31/1000*(1-Assumptions!$B$32*(1-Assumptions!$B$33))</f>
+        <f>Assumptions!$B$54*Assumptions!$B$34/1000*(1-Assumptions!$B$37*(1-Assumptions!$B$38))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Ad revenue per active day</t>
+          <t>Interstitial revenue per active day</t>
         </is>
       </c>
       <c r="B6" s="13">
-        <f>B4+B5</f>
+        <f>Assumptions!$B$36*Assumptions!$B$35/1000*(1-Assumptions!$B$37*(1-Assumptions!$B$38))</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>C4+C5</f>
+        <f>Assumptions!$B$36*Assumptions!$B$35/1000*(1-Assumptions!$B$37*(1-Assumptions!$B$38))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>AI cost without the budget cap</t>
+          <t>Ad revenue per active day</t>
         </is>
       </c>
       <c r="B7" s="13">
-        <f>Assumptions!$B$39*('Feature cost'!$B$5+'Feature cost'!$B$6)+Assumptions!$B$40*'Feature cost'!$B$4+Assumptions!$B$41*'Feature cost'!$B$7+Assumptions!$B$42*'Feature cost'!$B$8</f>
+        <f>B4+B5+B6</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>Assumptions!$B$45*('Feature cost'!$B$5+'Feature cost'!$B$6)+Assumptions!$B$46*'Feature cost'!$B$4+Assumptions!$B$47*'Feature cost'!$B$7+Assumptions!$B$48*'Feature cost'!$B$8</f>
+        <f>C4+C5+C6</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Daily AI budget (base + videos, capped)</t>
+          <t>AI cost without the budget cap</t>
         </is>
       </c>
       <c r="B8" s="13">
-        <f>Assumptions!$B$35+MIN(Assumptions!$B$43,Assumptions!$B$37)*Assumptions!$B$36</f>
+        <f>Assumptions!$B$44*('Feature cost'!$B$5+'Feature cost'!$B$6)+Assumptions!$B$45*'Feature cost'!$B$4+Assumptions!$B$46*'Feature cost'!$B$7+Assumptions!$B$47*'Feature cost'!$B$8</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>Assumptions!$B$35+MIN(Assumptions!$B$49,Assumptions!$B$37)*Assumptions!$B$36</f>
+        <f>Assumptions!$B$50*('Feature cost'!$B$5+'Feature cost'!$B$6)+Assumptions!$B$51*'Feature cost'!$B$4+Assumptions!$B$52*'Feature cost'!$B$7+Assumptions!$B$53*'Feature cost'!$B$8</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>AI cost per active day (after the cap; the plan always runs)</t>
+          <t>Daily AI budget (base + videos, capped)</t>
         </is>
       </c>
       <c r="B9" s="13">
-        <f>MIN(B7,MAX(B8,Assumptions!$B$39*('Feature cost'!$B$5+'Feature cost'!$B$6)))</f>
+        <f>Assumptions!$B$40+MIN(Assumptions!$B$48,Assumptions!$B$42)*Assumptions!$B$41</f>
         <v/>
       </c>
       <c r="C9" s="13">
-        <f>MIN(C7,MAX(C8,Assumptions!$B$45*('Feature cost'!$B$5+'Feature cost'!$B$6)))</f>
+        <f>Assumptions!$B$40+MIN(Assumptions!$B$54,Assumptions!$B$42)*Assumptions!$B$41</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Contribution per active day</t>
+          <t>AI cost per active day (after the cap; the plan always runs)</t>
         </is>
       </c>
       <c r="B10" s="13">
-        <f>B6-B9</f>
+        <f>MIN(B8,MAX(B9,Assumptions!$B$44*('Feature cost'!$B$5+'Feature cost'!$B$6)))</f>
         <v/>
       </c>
       <c r="C10" s="13">
-        <f>C6-C9</f>
+        <f>MIN(C8,MAX(C9,Assumptions!$B$50*('Feature cost'!$B$5+'Feature cost'!$B$6)))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>Contribution per active day</t>
+        </is>
+      </c>
+      <c r="B11" s="13">
+        <f>B7-B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="13">
+        <f>C7-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
           <t>Margin per active day</t>
         </is>
       </c>
-      <c r="B11" s="14">
-        <f>IF(B6=0,0,B10/B6)</f>
-        <v/>
-      </c>
-      <c r="C11" s="14">
-        <f>IF(C6=0,0,C10/C6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="B12" s="14">
+        <f>IF(B7=0,0,B11/B7)</f>
+        <v/>
+      </c>
+      <c r="C12" s="14">
+        <f>IF(C7=0,0,C11/C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Per month</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Ad revenue per month</t>
-        </is>
-      </c>
-      <c r="B13" s="15">
-        <f>B6*Assumptions!$B$51</f>
-        <v/>
-      </c>
-      <c r="C13" s="15">
-        <f>C6*Assumptions!$B$51</f>
-        <v/>
-      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>AI cost per month</t>
+          <t>Ad revenue per month</t>
         </is>
       </c>
       <c r="B14" s="15">
-        <f>B9*Assumptions!$B$51</f>
+        <f>B7*Assumptions!$B$56</f>
         <v/>
       </c>
       <c r="C14" s="15">
-        <f>C9*Assumptions!$B$51</f>
+        <f>C7*Assumptions!$B$56</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure per month</t>
+          <t>AI cost per month</t>
         </is>
       </c>
       <c r="B15" s="15">
-        <f>Assumptions!$B$52</f>
+        <f>B10*Assumptions!$B$56</f>
         <v/>
       </c>
       <c r="C15" s="15">
-        <f>Assumptions!$B$52</f>
+        <f>C10*Assumptions!$B$56</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Contribution per month</t>
+          <t>Infrastructure per month</t>
         </is>
       </c>
       <c r="B16" s="15">
-        <f>B13-B14-B15</f>
+        <f>Assumptions!$B$57</f>
         <v/>
       </c>
       <c r="C16" s="15">
-        <f>C13-C14-C15</f>
+        <f>Assumptions!$B$57</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Margin per month</t>
-        </is>
-      </c>
-      <c r="B17" s="14">
-        <f>IF(B13=0,0,B16/B13)</f>
-        <v/>
-      </c>
-      <c r="C17" s="14">
-        <f>IF(C13=0,0,C16/C13)</f>
+          <t>Contribution per month</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>B14-B15-B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="15">
+        <f>C14-C15-C16</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>Margin per month</t>
+        </is>
+      </c>
+      <c r="B18" s="14">
+        <f>IF(B14=0,0,B17/B14)</f>
+        <v/>
+      </c>
+      <c r="C18" s="14">
+        <f>IF(C14=0,0,C17/C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>Months of contribution to pay one SMS sign-up code</t>
         </is>
       </c>
-      <c r="B18" s="16">
-        <f>IF(B16&lt;=0,"never",Assumptions!$B$53/B16)</f>
-        <v/>
-      </c>
-      <c r="C18" s="16">
-        <f>IF(C16&lt;=0,"never",Assumptions!$B$53/C16)</f>
+      <c r="B19" s="16">
+        <f>IF(B17&lt;=0,"never",Assumptions!$B$58/B17)</f>
+        <v/>
+      </c>
+      <c r="C19" s="16">
+        <f>IF(C17&lt;=0,"never",Assumptions!$B$58/C17)</f>
         <v/>
       </c>
     </row>
@@ -1733,7 +1823,7 @@
         </is>
       </c>
       <c r="B3" s="17">
-        <f>Assumptions!$B$55*(1-Assumptions!$B$56)</f>
+        <f>Assumptions!$B$60*(1-Assumptions!$B$61)</f>
         <v/>
       </c>
     </row>
@@ -1744,7 +1834,7 @@
         </is>
       </c>
       <c r="B4" s="17">
-        <f>Assumptions!$B$58*Assumptions!$B$59*'Feature cost'!$C$4</f>
+        <f>Assumptions!$B$63*Assumptions!$B$64*'Feature cost'!$C$4</f>
         <v/>
       </c>
     </row>
@@ -1755,7 +1845,7 @@
         </is>
       </c>
       <c r="B5" s="17">
-        <f>Assumptions!$B$58*Assumptions!$B$60</f>
+        <f>Assumptions!$B$63*Assumptions!$B$65</f>
         <v/>
       </c>
     </row>
@@ -1777,7 +1867,7 @@
         </is>
       </c>
       <c r="B7" s="17">
-        <f>'Free user P&amp;L'!$B$16</f>
+        <f>'Free user P&amp;L'!$B$17</f>
         <v/>
       </c>
     </row>
@@ -1788,7 +1878,7 @@
         </is>
       </c>
       <c r="B8" s="17">
-        <f>Assumptions!$B$57*B6+(1-Assumptions!$B$57)*B7</f>
+        <f>Assumptions!$B$62*B6+(1-Assumptions!$B$62)*B7</f>
         <v/>
       </c>
     </row>
@@ -1799,7 +1889,7 @@
         </is>
       </c>
       <c r="B9" s="17">
-        <f>Assumptions!$B$57*B6</f>
+        <f>Assumptions!$B$62*B6</f>
         <v/>
       </c>
     </row>
@@ -1810,7 +1900,7 @@
         </is>
       </c>
       <c r="B10" s="17">
-        <f>(1-Assumptions!$B$57)*B7</f>
+        <f>(1-Assumptions!$B$62)*B7</f>
         <v/>
       </c>
     </row>
@@ -1851,40 +1941,40 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>'Free user P&amp;L'!$B$9</f>
+        <f>'Free user P&amp;L'!$B$10</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Banner revenue per active day</t>
+          <t>Banner + interstitial revenue per active day</t>
         </is>
       </c>
       <c r="B4" s="12">
-        <f>'Free user P&amp;L'!$B$4</f>
+        <f>'Free user P&amp;L'!$B$4+'Free user P&amp;L'!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Rewarded eCPM needed to cover AI (at this banner rate)</t>
+          <t>Rewarded eCPM needed to cover AI (at these banner and interstitial rates)</t>
         </is>
       </c>
       <c r="B5" s="17">
-        <f>IF(Assumptions!$B$43=0,0,MAX(0,(B3-B4))/Assumptions!$B$43*1000/(1-Assumptions!$B$32*(1-Assumptions!$B$33)))</f>
+        <f>IF(Assumptions!$B$48=0,0,MAX(0,(B3-B4))/Assumptions!$B$48*1000/(1-Assumptions!$B$37*(1-Assumptions!$B$38)))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Banner eCPM needed with no rewarded videos</t>
+          <t>Banner eCPM needed with no rewarded videos or interstitials</t>
         </is>
       </c>
       <c r="B6" s="17">
-        <f>IF(Assumptions!$B$30=0,0,B3/Assumptions!$B$30*1000/(1-Assumptions!$B$32*(1-Assumptions!$B$33)))</f>
+        <f>IF(Assumptions!$B$33=0,0,B3/Assumptions!$B$33*1000/(1-Assumptions!$B$37*(1-Assumptions!$B$38)))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: bot protection, per-user limits, data retention, lower free AI budget
- Cloudflare Turnstile CAPTCHA on sign-up, password sign-in, code resends
  and password resets (off until a site key is configured)
- send-sms: EU/EEA/UK/CH calling codes only, caps per number and overall
  with HMAC-keyed counters; fails closed
- Per-user caps on food-search and food-barcode (rate_limit_hit)
- purge_old_data(): retention periods from app_config, health log kept
- Free AI budget $0.04 -> $0.03 a day
- Adds react-native-webview (CAPTCHA), expo-store-review and
  expo-tracking-transparency (used next)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FhfEYVk2hN2wqZc7JaLb6E
</commit_message>
<xml_diff>
--- a/docs/business/ai-ad-economics.xlsx
+++ b/docs/business/ai-ad-economics.xlsx
@@ -1009,11 +1009,11 @@
         </is>
       </c>
       <c r="B40" s="11" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>ai_free_daily_budget_usd: a backstop sized to the free allowance</t>
+          <t>ai_free_daily_budget_usd: a backstop (overnight batch plans do not count)</t>
         </is>
       </c>
     </row>

</xml_diff>